<commit_message>
Finished adding DC-DC Converters - Isolated table to database
</commit_message>
<xml_diff>
--- a/To Add v2/PSUs - PCB Mount - DC-DC - Isolated.xlsx
+++ b/To Add v2/PSUs - PCB Mount - DC-DC - Isolated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312CDB43-C04F-42A7-9BDD-B85C3D5DF88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B53CC10-475D-410F-929F-42E75FCA5D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Remember to modify the Kicad DBL!!!</t>
   </si>
@@ -99,12 +99,6 @@
   </si>
   <si>
     <t>Complete?</t>
-  </si>
-  <si>
-    <t>Generate w/ concact</t>
-  </si>
-  <si>
-    <t>Foobar</t>
   </si>
   <si>
     <t>DB Params</t>
@@ -514,13 +508,17 @@
   <dimension ref="B1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.81640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.1796875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.7265625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.08984375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.81640625" customWidth="1"/>
     <col min="15" max="15" width="9.6328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.36328125" customWidth="1"/>
     <col min="18" max="18" width="21" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="20" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="15" bestFit="1" customWidth="1"/>
@@ -710,28 +708,28 @@
         <v>9</v>
       </c>
       <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" t="s">
         <v>25</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>26</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>27</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
         <v>28</v>
       </c>
-      <c r="I6" t="s">
+      <c r="L6" t="s">
         <v>29</v>
-      </c>
-      <c r="J6" t="s">
-        <v>36</v>
-      </c>
-      <c r="K6" t="s">
-        <v>30</v>
-      </c>
-      <c r="L6" t="s">
-        <v>31</v>
       </c>
       <c r="M6" t="s">
         <v>10</v>
@@ -768,59 +766,61 @@
       </c>
     </row>
     <row r="7" spans="2:28" x14ac:dyDescent="0.35">
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
+      <c r="C7" t="str">
+        <f>_xlfn.CONCAT(E7,"out ",G7," ",F7,"in ",H7," ",L7," ",J7," ",K7," ",I7)</f>
+        <v>3.3/5Vout 200mA 3-5.5Vin 2121Vpk 26MHz 0.505 5pF SMD</v>
+      </c>
+      <c r="D7" t="str">
+        <f>_xlfn.CONCAT(F7," to ",E7," ",G7)</f>
+        <v>3-5.5V to 3.3/5V 200mA</v>
       </c>
       <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
         <v>37</v>
       </c>
-      <c r="F7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" t="s">
-        <v>39</v>
-      </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J7" s="2">
         <v>0.505</v>
       </c>
       <c r="K7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="M7" t="s">
+        <v>31</v>
+      </c>
+      <c r="N7" t="s">
+        <v>30</v>
+      </c>
+      <c r="O7" t="s">
+        <v>22</v>
+      </c>
+      <c r="P7" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q7" t="s">
         <v>33</v>
       </c>
-      <c r="N7" t="s">
-        <v>32</v>
-      </c>
-      <c r="O7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P7" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>35</v>
-      </c>
       <c r="R7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="S7" t="s">
+        <v>42</v>
+      </c>
+      <c r="T7" t="s">
         <v>44</v>
-      </c>
-      <c r="T7" t="s">
-        <v>46</v>
       </c>
       <c r="W7">
         <f>COUNTBLANK(C7:T7)</f>
@@ -835,7 +835,7 @@
         <v>1</v>
       </c>
       <c r="AA7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AB7">
         <f>SUM(C4:T4)</f>

</xml_diff>

<commit_message>
Added RFM-0505S to database
</commit_message>
<xml_diff>
--- a/To Add v2/PSUs - PCB Mount - DC-DC - Isolated.xlsx
+++ b/To Add v2/PSUs - PCB Mount - DC-DC - Isolated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B53CC10-475D-410F-929F-42E75FCA5D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B7B5E10-B245-4018-A493-D6F7E0BD51B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="7725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
   <si>
     <t>Remember to modify the Kicad DBL!!!</t>
   </si>
@@ -171,6 +171,36 @@
   </si>
   <si>
     <t> </t>
+  </si>
+  <si>
+    <t>https://recom-power.com/pdf/Econoline/RFM.pdf</t>
+  </si>
+  <si>
+    <t>5V</t>
+  </si>
+  <si>
+    <t>500Vpk</t>
+  </si>
+  <si>
+    <t>ThruHole</t>
+  </si>
+  <si>
+    <t>75pF</t>
+  </si>
+  <si>
+    <t>80kHz</t>
+  </si>
+  <si>
+    <t>RFM-0505S</t>
+  </si>
+  <si>
+    <t>945-3159-ND</t>
+  </si>
+  <si>
+    <t>0Dan_PSUs:DC-DC_2pI_2pO_invpol</t>
+  </si>
+  <si>
+    <t>DCDC_ISO:Recom_RFM</t>
   </si>
 </sst>
 </file>
@@ -213,10 +243,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -505,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AB7"/>
+  <dimension ref="B1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="50.1796875" bestFit="1" customWidth="1"/>
@@ -538,75 +569,75 @@
       </c>
       <c r="C2">
         <f>COUNTA(C7:C9999)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:T2" si="0">COUNTA(D7:D9999)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
         <f t="shared" ref="F2:L2" si="1">COUNTA(F7:F9999)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
         <f t="shared" ref="J2" si="2">COUNTA(J7:J9999)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA2" t="s">
         <v>3</v>
@@ -622,7 +653,7 @@
       </c>
       <c r="AB3">
         <f>MAX(C2:T2)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="2:28" x14ac:dyDescent="0.35">
@@ -688,7 +719,7 @@
       </c>
       <c r="AB4">
         <f>SUM(Y7:Y9999)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:28" x14ac:dyDescent="0.35">
@@ -840,6 +871,76 @@
       <c r="AB7">
         <f>SUM(C4:T4)</f>
         <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="2:28" x14ac:dyDescent="0.35">
+      <c r="C8" t="str">
+        <f>_xlfn.CONCAT(E8,"out ",G8," ",F8,"in ",H8," ",L8," ",J8," ",K8," ",I8)</f>
+        <v>5Vout 200mA 5Vin 500Vpk 80kHz 0.79 75pF ThruHole</v>
+      </c>
+      <c r="D8" t="str">
+        <f>_xlfn.CONCAT(F8," to ",E8," ",G8)</f>
+        <v>5V to 5V 200mA</v>
+      </c>
+      <c r="E8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="3">
+        <v>0.79</v>
+      </c>
+      <c r="K8" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" t="s">
+        <v>50</v>
+      </c>
+      <c r="M8" t="s">
+        <v>31</v>
+      </c>
+      <c r="N8" t="s">
+        <v>51</v>
+      </c>
+      <c r="O8" t="s">
+        <v>22</v>
+      </c>
+      <c r="P8" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>45</v>
+      </c>
+      <c r="R8" t="s">
+        <v>53</v>
+      </c>
+      <c r="S8" t="s">
+        <v>54</v>
+      </c>
+      <c r="T8" t="s">
+        <v>44</v>
+      </c>
+      <c r="W8">
+        <f>COUNTBLANK(C8:T8)</f>
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <f>100*COUNTA(C8:T8)/$AB$7</f>
+        <v>100</v>
+      </c>
+      <c r="Y8">
+        <f>IF(X8=100,1,0)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>